<commit_message>
corrected tales of phantasia psx entries
</commit_message>
<xml_diff>
--- a/Docs/Missing Games (26 December 2025).xlsx
+++ b/Docs/Missing Games (26 December 2025).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Unofficial-RA-DATs\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ACC72FC-22D7-4485-A149-B020945F78F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27848846-D9A1-4BAF-A7C9-CC636DE24BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="12" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1 - Sega Genesis" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="951" uniqueCount="624">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="954" uniqueCount="627">
   <si>
     <t>GAME NAME</t>
   </si>
@@ -1913,6 +1913,15 @@
   </si>
   <si>
     <t>Can't find the rom/patch for this game.</t>
+  </si>
+  <si>
+    <t>Tales of Phantasia (Japan) (En) (v1.0) (Absolute Zero)</t>
+  </si>
+  <si>
+    <t>5864d666f93bd1a24af232f7bfefb53b</t>
+  </si>
+  <si>
+    <t>Game doesn't boot up past a black screen.</t>
   </si>
 </sst>
 </file>
@@ -7752,7 +7761,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12EA685A-6B74-42D3-8C63-E13E4551FD07}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="56.7109375" bestFit="1" customWidth="1"/>
@@ -7780,6 +7789,17 @@
       </c>
       <c r="C2" t="s">
         <v>577</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>624</v>
+      </c>
+      <c r="B3" t="s">
+        <v>625</v>
+      </c>
+      <c r="C3" t="s">
+        <v>626</v>
       </c>
     </row>
   </sheetData>

</xml_diff>